<commit_message>
Feat: Implement Task Wizard with Excel Import
</commit_message>
<xml_diff>
--- a/260303-workers list.xlsx
+++ b/260303-workers list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\aiagent\worker_view_cal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6647AFF-5CF4-41CA-B038-4E810FF6745E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{349DE45E-9E3A-4A23-B6BC-18A21D946642}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" activeTab="1" xr2:uid="{18B37074-D316-4EE9-80CC-81AEDE942E64}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="79">
   <si>
     <t>陳易璘</t>
   </si>
@@ -322,6 +322,14 @@
   </si>
   <si>
     <t>傑</t>
+  </si>
+  <si>
+    <t>紅色</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>灰色</t>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1294,7 +1302,7 @@
         <v>69</v>
       </c>
       <c r="D2" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -1308,7 +1316,7 @@
         <v>69</v>
       </c>
       <c r="D3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -1322,7 +1330,7 @@
         <v>67</v>
       </c>
       <c r="D4" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Feat: Add shift time and copy to clipboard schedule
</commit_message>
<xml_diff>
--- a/260303-workers list.xlsx
+++ b/260303-workers list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\aiagent\worker_view_cal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{349DE45E-9E3A-4A23-B6BC-18A21D946642}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{564EA9A5-BD9C-46A7-BB2A-EE4F1D68B7DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" activeTab="1" xr2:uid="{18B37074-D316-4EE9-80CC-81AEDE942E64}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{18B37074-D316-4EE9-80CC-81AEDE942E64}"/>
   </bookViews>
   <sheets>
     <sheet name="工班清單" sheetId="1" r:id="rId1"/>
@@ -89,10 +89,6 @@
     <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
-    <t>旻</t>
-    <phoneticPr fontId="9" type="noConversion"/>
-  </si>
-  <si>
     <t>李祐緯</t>
     <phoneticPr fontId="9" type="noConversion"/>
   </si>
@@ -330,6 +326,9 @@
   <si>
     <t>灰色</t>
     <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>揆</t>
   </si>
 </sst>
 </file>
@@ -963,10 +962,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -1021,7 +1020,7 @@
         <v>16</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>17</v>
+        <v>78</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -1029,10 +1028,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
@@ -1040,10 +1039,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
@@ -1051,10 +1050,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
@@ -1062,10 +1061,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
@@ -1073,10 +1072,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
@@ -1084,10 +1083,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
@@ -1095,10 +1094,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
@@ -1106,10 +1105,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
+        <v>69</v>
+      </c>
+      <c r="C17" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
@@ -1117,10 +1116,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
@@ -1128,10 +1127,10 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
+        <v>31</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>32</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
@@ -1139,10 +1138,10 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
+        <v>33</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
@@ -1153,7 +1152,7 @@
         <v>6</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
@@ -1161,10 +1160,10 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
@@ -1172,10 +1171,10 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
@@ -1279,184 +1278,184 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>41</v>
       </c>
-      <c r="C1" t="s">
-        <v>42</v>
-      </c>
       <c r="D1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C8" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D8" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C10" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B12" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="C12" t="s">
         <v>65</v>
       </c>
-      <c r="C12" t="s">
-        <v>66</v>
-      </c>
       <c r="D12" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C13" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>